<commit_message>
new installer with improved Z line metrics
</commit_message>
<xml_diff>
--- a/demo/demo_analysis_across.xlsx
+++ b/demo/demo_analysis_across.xlsx
@@ -204,13 +204,13 @@
         <v>1</v>
       </c>
       <c r="D2" s="0">
-        <v>1.7377738872517052</v>
+        <v>1.7397782400628372</v>
       </c>
       <c r="E2" s="0">
-        <v>0.04990798251508255</v>
+        <v>0.049907982515077658</v>
       </c>
       <c r="F2" s="0">
-        <v>0.022319528304719099</v>
+        <v>0.022319528304716913</v>
       </c>
       <c r="G2" s="0">
         <v>1.0504373099468038</v>
@@ -255,7 +255,7 @@
         <v>1</v>
       </c>
       <c r="C2" s="0">
-        <v>1.7437869456851187</v>
+        <v>1.7036998894624729</v>
       </c>
     </row>
     <row r="3">
@@ -266,7 +266,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="0">
-        <v>1.8039175300190584</v>
+        <v>1.8239610581303791</v>
       </c>
     </row>
     <row r="4">
@@ -277,7 +277,7 @@
         <v>3</v>
       </c>
       <c r="C4" s="0">
-        <v>1.7337651816294344</v>
+        <v>1.7237434175737816</v>
       </c>
     </row>
     <row r="5">
@@ -288,7 +288,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="0">
-        <v>1.7437869456851018</v>
+        <v>1.7437869456850965</v>
       </c>
     </row>
     <row r="6">
@@ -299,7 +299,7 @@
         <v>5</v>
       </c>
       <c r="C6" s="0">
-        <v>1.663612833239813</v>
+        <v>1.7036998894624556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>